<commit_message>
Rename hats snood product type
</commit_message>
<xml_diff>
--- a/app/download_dir/system_files/шляпы_по каждому размеру.xlsx
+++ b/app/download_dir/system_files/шляпы_по каждому размеру.xlsx
@@ -14600,7 +14600,7 @@
     <row r="33" ht="13.8" customHeight="1" s="68">
       <c r="D33" s="41" t="inlineStr">
         <is>
-          <t>СНУД</t>
+          <t>ШАРФ-СНУД</t>
         </is>
       </c>
       <c r="E33" s="41" t="inlineStr">
@@ -16641,7 +16641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:E110"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.83984375" defaultRowHeight="12.8" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="19.77" customWidth="1" style="41" min="2" max="2"/>
@@ -16650,6 +16650,7 @@
     <col width="29.63" customWidth="1" style="41" min="5" max="5"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="12.8" customHeight="1" s="68">
       <c r="B2" s="74" t="inlineStr">
         <is>
@@ -17799,7 +17800,7 @@
     <row r="33" ht="40.25" customFormat="1" customHeight="1" s="76">
       <c r="A33" s="79" t="inlineStr">
         <is>
-          <t>&lt;4070000032&gt; СНУД</t>
+          <t>&lt;4070000032&gt; ШАРФ-СНУД</t>
         </is>
       </c>
       <c r="B33" s="80" t="n"/>

</xml_diff>